<commit_message>
feat: implement bulk material import via Excel with queued processing and data management controllers
</commit_message>
<xml_diff>
--- a/public/excel/Material-template.xlsx
+++ b/public/excel/Material-template.xlsx
@@ -1,26 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Academics\Capstone\BPS-LMS-Admin\public\excel\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0522167C-0614-43E3-8F63-EC0197B8FD78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Import Template" sheetId="1" r:id="rId1"/>
+    <sheet name="Import Template" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="44">
+  <si>
+    <t>SNCS-LMS MATERIAL IMPORT TEMPLATE</t>
+  </si>
   <si>
     <t>IMPORT INSTRUCTIONS:</t>
   </si>
@@ -145,49 +143,71 @@
     <t>Literature; Fiction</t>
   </si>
   <si>
-    <t>SNCS-LMS MATERIAL IMPORT TEMPLATE</t>
+    <t>Parallel Title</t>
+  </si>
+  <si>
+    <t>Series</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
+  <fonts count="6">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <i/>
+      <b val="0"/>
+      <i val="1"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="16"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -238,32 +258,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="2" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="3" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -553,16 +565,44 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:Z19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="24" width="20" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="true" style="0"/>
+    <col min="2" max="2" width="20" customWidth="true" style="0"/>
+    <col min="3" max="3" width="20" customWidth="true" style="0"/>
+    <col min="4" max="4" width="20" customWidth="true" style="0"/>
+    <col min="5" max="5" width="20" customWidth="true" style="0"/>
+    <col min="6" max="6" width="20" customWidth="true" style="0"/>
+    <col min="7" max="7" width="20" customWidth="true" style="0"/>
+    <col min="8" max="8" width="20" customWidth="true" style="0"/>
+    <col min="9" max="9" width="20" customWidth="true" style="0"/>
+    <col min="10" max="10" width="20" customWidth="true" style="0"/>
+    <col min="11" max="11" width="20" customWidth="true" style="0"/>
+    <col min="12" max="12" width="20" customWidth="true" style="0"/>
+    <col min="13" max="13" width="20" customWidth="true" style="0"/>
+    <col min="14" max="14" width="20" customWidth="true" style="0"/>
+    <col min="15" max="15" width="20" customWidth="true" style="0"/>
+    <col min="16" max="16" width="20" customWidth="true" style="0"/>
+    <col min="17" max="17" width="20" customWidth="true" style="0"/>
+    <col min="18" max="18" width="20" customWidth="true" style="0"/>
+    <col min="19" max="19" width="20" customWidth="true" style="0"/>
+    <col min="20" max="20" width="20" customWidth="true" style="0"/>
+    <col min="21" max="21" width="20" customWidth="true" style="0"/>
+    <col min="22" max="22" width="20" customWidth="true" style="0"/>
+    <col min="23" max="23" width="20" customWidth="true" style="0"/>
+    <col min="24" max="24" width="20" customWidth="true" style="0"/>
+    <col min="25" max="25" width="25" customWidth="true" style="0"/>
+    <col min="26" max="26" width="20" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:26" customHeight="1" ht="21">
       <c r="A1" s="6" t="s">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -590,7 +630,7 @@
       <c r="Y1" s="7"/>
       <c r="Z1" s="7"/>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -618,9 +658,9 @@
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
     </row>
-    <row r="3" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" customHeight="1" ht="15.6">
       <c r="A3" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -648,9 +688,9 @@
       <c r="Y3" s="3"/>
       <c r="Z3" s="3"/>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26">
       <c r="A4" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -678,9 +718,9 @@
       <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26">
       <c r="A5" s="4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -708,9 +748,9 @@
       <c r="Y5" s="3"/>
       <c r="Z5" s="3"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26">
       <c r="A6" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -738,9 +778,9 @@
       <c r="Y6" s="3"/>
       <c r="Z6" s="3"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26">
       <c r="A7" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -768,9 +808,9 @@
       <c r="Y7" s="3"/>
       <c r="Z7" s="3"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26">
       <c r="A8" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -798,9 +838,9 @@
       <c r="Y8" s="3"/>
       <c r="Z8" s="3"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26">
       <c r="A9" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -828,9 +868,9 @@
       <c r="Y9" s="3"/>
       <c r="Z9" s="3"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26">
       <c r="A10" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -858,9 +898,9 @@
       <c r="Y10" s="3"/>
       <c r="Z10" s="3"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26">
       <c r="A11" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -888,9 +928,9 @@
       <c r="Y11" s="3"/>
       <c r="Z11" s="3"/>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26">
       <c r="A12" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -918,9 +958,9 @@
       <c r="Y12" s="3"/>
       <c r="Z12" s="3"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26">
       <c r="A13" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -948,7 +988,7 @@
       <c r="Y13" s="3"/>
       <c r="Z13" s="3"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -976,7 +1016,7 @@
       <c r="Y14" s="1"/>
       <c r="Z14" s="1"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:26">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -1004,7 +1044,7 @@
       <c r="Y15" s="1"/>
       <c r="Z15" s="1"/>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:26">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -1032,7 +1072,7 @@
       <c r="Y16" s="1"/>
       <c r="Z16" s="1"/>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:26">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1060,102 +1100,108 @@
       <c r="Y17" s="1"/>
       <c r="Z17" s="1"/>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:26">
       <c r="A18" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L18" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N18" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O18" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P18" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q18" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R18" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S18" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="T18" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="U18" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="V18" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="W18" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="X18" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+      <c r="Y18" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z18" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:26">
       <c r="A19" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B19" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="U19" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="V19" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="X19" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells>
     <mergeCell ref="A12:Z12"/>
     <mergeCell ref="A13:Z13"/>
     <mergeCell ref="A7:Z7"/>
@@ -1169,6 +1215,8 @@
     <mergeCell ref="A5:Z5"/>
     <mergeCell ref="A6:Z6"/>
   </mergeCells>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
 </worksheet>
 </file>
</xml_diff>